<commit_message>
Import d'inventaire : colonne Note/Commentaire, CSV à virgule décimale ; version 67
- Colonne Note (Note, Commentaire, Observation, Obs, Remarque, Rem)
  reprise dans le commentaire du billon importé.
- CSV lu en texte brut : « 8,20 » n'est plus lu 820 m ; encodage UTF-8
  ou Windows-1252 (CSV d'Excel en français), réductions à virgule.
- Manuel terrain 3.12 et modèle Excel mis à jour (colonne note).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0198enRLQRZEqawz6FFmpXkK
</commit_message>
<xml_diff>
--- a/manuels/modele-import-inventaire.xlsx
+++ b/manuels/modele-import-inventaire.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -434,6 +434,7 @@
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -472,6 +473,11 @@
           <t>reduction_d</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -516,6 +522,11 @@
       </c>
       <c r="F3" t="n">
         <v>100</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>gélivure</t>
+        </is>
       </c>
     </row>
     <row r="4">

</xml_diff>